<commit_message>
Add January and February sheets; quarter sums from months.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/creer-une-skill/Budget_vs_Realise_AlpesConseil.xlsx
+++ b/creer-une-skill/Budget_vs_Realise_AlpesConseil.xlsx
@@ -8,9 +8,11 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consignes" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mars" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trimestre" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corrige_formateur" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Janvier" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fevrier" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mars" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trimestre" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Corrige_formateur" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -515,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -538,7 +540,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Utilisez la feuille « Mars » (ou « Trimestre ») avec votre skill budget-variance-note. Demandez à Claude / Cursor : « Rédige la note d'écarts à partir de ce fichier ». La skill doit produire synthèse, tableau des 3 postes clés, questions métier et une prochaine action.</t>
+          <t>Utilisez la feuille « Mars » (ou « Trimestre ») avec votre skill budget-variance-note. Demandez à Claude / Cursor : « Rédige la note d'écarts à partir de ce fichier ». La skill doit produire synthèse, tableau des 3 postes clés, questions métier et une prochaine action. Janvier et Février permettent d’expliquer le trimestre.</t>
         </is>
       </c>
     </row>
@@ -561,28 +563,28 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>2. Ouvrez ce classeur — ne lisez que la feuille Mars pour le premier essai.</t>
+          <t>2. Ouvrez ce classeur — premier essai : feuille Mars seulement.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>3. Lancez la skill sur les chiffres de Mars (sans regarder la feuille Corrigé).</t>
+          <t>3. Lancez la skill sur les chiffres de Mars (sans regarder Corrige_formateur).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>4. Comparez votre note à la feuille Corrigé_formateur (ordre de grandeur, pas mot à mot).</t>
+          <t>4. Comparez votre note à Corrige_formateur (ordre de grandeur, pas mot à mot).</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>5. Variante : refaites l'exercice avec la feuille Trimestre.</t>
+          <t>5. Variante : feuille Trimestre (somme Janvier + Février + Mars), puis explorez les mois.</t>
         </is>
       </c>
     </row>
@@ -597,6 +599,20 @@
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Alpes Conseil Sàrl — cabinet de conseil, Vaud. Devise : CHF. Fichier pédagogique uniquement — pas de conseil fiscal ou financier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Cohérence des chiffres</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>La feuille Trimestre additionne Janvier + Février + Mars (formules). Modifier un mois met à jour le trimestre.</t>
         </is>
       </c>
     </row>
@@ -610,6 +626,662 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Alpes Conseil Sàrl — Budget vs réalisé</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Période : janvier 2026  |  Comparaison : budget mensuel vs réalisé</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Poste</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Budget CHF</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Réalisé CHF</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Écart CHF</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Écart %</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Commentaire métier (brut)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Chiffre d'affaires — honoraires</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="n">
+        <v>88000</v>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>86000</v>
+      </c>
+      <c r="D5" s="8">
+        <f>C5-B5</f>
+        <v/>
+      </c>
+      <c r="E5" s="9">
+        <f>IF(B5=0,0,D5/B5)</f>
+        <v/>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>Démarrage année : pipeline correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Autres produits</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>1900</v>
+      </c>
+      <c r="D6" s="11">
+        <f>C6-B6</f>
+        <v/>
+      </c>
+      <c r="E6" s="12">
+        <f>IF(B6=0,0,D6/B6)</f>
+        <v/>
+      </c>
+      <c r="F6" s="10" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Charges de personnel</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="n">
+        <v>55000</v>
+      </c>
+      <c r="C7" s="8" t="n">
+        <v>55200</v>
+      </c>
+      <c r="D7" s="8">
+        <f>C7-B7</f>
+        <v/>
+      </c>
+      <c r="E7" s="9">
+        <f>IF(B7=0,0,D7/B7)</f>
+        <v/>
+      </c>
+      <c r="F7" s="7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>Sous-traitance / freelances</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="n">
+        <v>8000</v>
+      </c>
+      <c r="C8" s="11" t="n">
+        <v>9000</v>
+      </c>
+      <c r="D8" s="11">
+        <f>C8-B8</f>
+        <v/>
+      </c>
+      <c r="E8" s="12">
+        <f>IF(B8=0,0,D8/B8)</f>
+        <v/>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>Pic ponctuel sur une mission</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Loyer et charges locatives</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="n">
+        <v>4500</v>
+      </c>
+      <c r="C9" s="8" t="n">
+        <v>4500</v>
+      </c>
+      <c r="D9" s="8">
+        <f>C9-B9</f>
+        <v/>
+      </c>
+      <c r="E9" s="9">
+        <f>IF(B9=0,0,D9/B9)</f>
+        <v/>
+      </c>
+      <c r="F9" s="7" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Marketing et acquisition</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C10" s="11" t="n">
+        <v>3400</v>
+      </c>
+      <c r="D10" s="11">
+        <f>C10-B10</f>
+        <v/>
+      </c>
+      <c r="E10" s="12">
+        <f>IF(B10=0,0,D10/B10)</f>
+        <v/>
+      </c>
+      <c r="F10" s="10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Informatique / outils</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="n">
+        <v>1800</v>
+      </c>
+      <c r="C11" s="8" t="n">
+        <v>1700</v>
+      </c>
+      <c r="D11" s="8">
+        <f>C11-B11</f>
+        <v/>
+      </c>
+      <c r="E11" s="9">
+        <f>IF(B11=0,0,D11/B11)</f>
+        <v/>
+      </c>
+      <c r="F11" s="7" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>Autres frais généraux</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="n">
+        <v>2700</v>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>2700</v>
+      </c>
+      <c r="D12" s="11">
+        <f>C12-B12</f>
+        <v/>
+      </c>
+      <c r="E12" s="12">
+        <f>IF(B12=0,0,D12/B12)</f>
+        <v/>
+      </c>
+      <c r="F12" s="10" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>Total produits</t>
+        </is>
+      </c>
+      <c r="B14" s="14">
+        <f>B5+B6</f>
+        <v/>
+      </c>
+      <c r="C14" s="14">
+        <f>C5+C6</f>
+        <v/>
+      </c>
+      <c r="D14" s="14">
+        <f>C14-B14</f>
+        <v/>
+      </c>
+      <c r="E14" s="15">
+        <f>IF(B14=0,0,D14/B14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>Total charges</t>
+        </is>
+      </c>
+      <c r="B15" s="14">
+        <f>SUM(B7:B12)</f>
+        <v/>
+      </c>
+      <c r="C15" s="14">
+        <f>SUM(C7:C12)</f>
+        <v/>
+      </c>
+      <c r="D15" s="14">
+        <f>C15-B15</f>
+        <v/>
+      </c>
+      <c r="E15" s="15">
+        <f>IF(B15=0,0,D15/B15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>Résultat d'exploitation (approx.)</t>
+        </is>
+      </c>
+      <c r="B16" s="14">
+        <f>B14-B15</f>
+        <v/>
+      </c>
+      <c r="C16" s="14">
+        <f>C14-C15</f>
+        <v/>
+      </c>
+      <c r="D16" s="14">
+        <f>C16-B16</f>
+        <v/>
+      </c>
+      <c r="E16" s="15">
+        <f>IF(B16=0,0,D16/B16)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Alpes Conseil Sàrl — Budget vs réalisé</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Période : février 2026  |  Comparaison : budget mensuel vs réalisé</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>Poste</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Budget CHF</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>Réalisé CHF</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>Écart CHF</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Écart %</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>Commentaire métier (brut)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>Chiffre d'affaires — honoraires</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="n">
+        <v>92000</v>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>83000</v>
+      </c>
+      <c r="D5" s="8">
+        <f>C5-B5</f>
+        <v/>
+      </c>
+      <c r="E5" s="9">
+        <f>IF(B5=0,0,D5/B5)</f>
+        <v/>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>1 mission décalée en mars</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Autres produits</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C6" s="11" t="n">
+        <v>1800</v>
+      </c>
+      <c r="D6" s="11">
+        <f>C6-B6</f>
+        <v/>
+      </c>
+      <c r="E6" s="12">
+        <f>IF(B6=0,0,D6/B6)</f>
+        <v/>
+      </c>
+      <c r="F6" s="10" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Charges de personnel</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="n">
+        <v>55000</v>
+      </c>
+      <c r="C7" s="8" t="n">
+        <v>56300</v>
+      </c>
+      <c r="D7" s="8">
+        <f>C7-B7</f>
+        <v/>
+      </c>
+      <c r="E7" s="9">
+        <f>IF(B7=0,0,D7/B7)</f>
+        <v/>
+      </c>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>Formation interne (heures non facturables)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>Sous-traitance / freelances</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="n">
+        <v>8000</v>
+      </c>
+      <c r="C8" s="11" t="n">
+        <v>10000</v>
+      </c>
+      <c r="D8" s="11">
+        <f>C8-B8</f>
+        <v/>
+      </c>
+      <c r="E8" s="12">
+        <f>IF(B8=0,0,D8/B8)</f>
+        <v/>
+      </c>
+      <c r="F8" s="10" t="inlineStr">
+        <is>
+          <t>Renfort sur livrable client clé</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Loyer et charges locatives</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="n">
+        <v>4500</v>
+      </c>
+      <c r="C9" s="8" t="n">
+        <v>4500</v>
+      </c>
+      <c r="D9" s="8">
+        <f>C9-B9</f>
+        <v/>
+      </c>
+      <c r="E9" s="9">
+        <f>IF(B9=0,0,D9/B9)</f>
+        <v/>
+      </c>
+      <c r="F9" s="7" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Marketing et acquisition</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C10" s="11" t="n">
+        <v>3900</v>
+      </c>
+      <c r="D10" s="11">
+        <f>C10-B10</f>
+        <v/>
+      </c>
+      <c r="E10" s="12">
+        <f>IF(B10=0,0,D10/B10)</f>
+        <v/>
+      </c>
+      <c r="F10" s="10" t="inlineStr">
+        <is>
+          <t>Sponsoring événement métier</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Informatique / outils</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="n">
+        <v>1800</v>
+      </c>
+      <c r="C11" s="8" t="n">
+        <v>1650</v>
+      </c>
+      <c r="D11" s="8">
+        <f>C11-B11</f>
+        <v/>
+      </c>
+      <c r="E11" s="9">
+        <f>IF(B11=0,0,D11/B11)</f>
+        <v/>
+      </c>
+      <c r="F11" s="7" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>Autres frais généraux</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="n">
+        <v>2700</v>
+      </c>
+      <c r="C12" s="11" t="n">
+        <v>2700</v>
+      </c>
+      <c r="D12" s="11">
+        <f>C12-B12</f>
+        <v/>
+      </c>
+      <c r="E12" s="12">
+        <f>IF(B12=0,0,D12/B12)</f>
+        <v/>
+      </c>
+      <c r="F12" s="10" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>Total produits</t>
+        </is>
+      </c>
+      <c r="B14" s="14">
+        <f>B5+B6</f>
+        <v/>
+      </c>
+      <c r="C14" s="14">
+        <f>C5+C6</f>
+        <v/>
+      </c>
+      <c r="D14" s="14">
+        <f>C14-B14</f>
+        <v/>
+      </c>
+      <c r="E14" s="15">
+        <f>IF(B14=0,0,D14/B14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="13" t="inlineStr">
+        <is>
+          <t>Total charges</t>
+        </is>
+      </c>
+      <c r="B15" s="14">
+        <f>SUM(B7:B12)</f>
+        <v/>
+      </c>
+      <c r="C15" s="14">
+        <f>SUM(C7:C12)</f>
+        <v/>
+      </c>
+      <c r="D15" s="14">
+        <f>C15-B15</f>
+        <v/>
+      </c>
+      <c r="E15" s="15">
+        <f>IF(B15=0,0,D15/B15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>Résultat d'exploitation (approx.)</t>
+        </is>
+      </c>
+      <c r="B16" s="14">
+        <f>B14-B15</f>
+        <v/>
+      </c>
+      <c r="C16" s="14">
+        <f>C14-C15</f>
+        <v/>
+      </c>
+      <c r="D16" s="14">
+        <f>C16-B16</f>
+        <v/>
+      </c>
+      <c r="E16" s="15">
+        <f>IF(B16=0,0,D16/B16)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -957,13 +1629,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -983,7 +1655,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Période : janvier–mars 2026  |  Variante pour un 2e essai</t>
+          <t>Période : janvier–mars 2026  |  Budget et réalisé = Janvier + Fevrier + Mars (formules)</t>
         </is>
       </c>
     </row>
@@ -1020,11 +1692,13 @@
           <t>Chiffre d'affaires — honoraires</t>
         </is>
       </c>
-      <c r="B5" s="8" t="n">
-        <v>280000</v>
-      </c>
-      <c r="C5" s="8" t="n">
-        <v>251000</v>
+      <c r="B5" s="8">
+        <f>Janvier!B5+Fevrier!B5+Mars!B5</f>
+        <v/>
+      </c>
+      <c r="C5" s="8">
+        <f>Janvier!C5+Fevrier!C5+Mars!C5</f>
+        <v/>
       </c>
       <c r="D5" s="8">
         <f>C5-B5</f>
@@ -1041,11 +1715,13 @@
           <t>Autres produits</t>
         </is>
       </c>
-      <c r="B6" s="11" t="n">
-        <v>6000</v>
-      </c>
-      <c r="C6" s="11" t="n">
-        <v>5200</v>
+      <c r="B6" s="11">
+        <f>Janvier!B6+Fevrier!B6+Mars!B6</f>
+        <v/>
+      </c>
+      <c r="C6" s="11">
+        <f>Janvier!C6+Fevrier!C6+Mars!C6</f>
+        <v/>
       </c>
       <c r="D6" s="11">
         <f>C6-B6</f>
@@ -1062,11 +1738,13 @@
           <t>Charges de personnel</t>
         </is>
       </c>
-      <c r="B7" s="8" t="n">
-        <v>165000</v>
-      </c>
-      <c r="C7" s="8" t="n">
-        <v>168000</v>
+      <c r="B7" s="8">
+        <f>Janvier!B7+Fevrier!B7+Mars!B7</f>
+        <v/>
+      </c>
+      <c r="C7" s="8">
+        <f>Janvier!C7+Fevrier!C7+Mars!C7</f>
+        <v/>
       </c>
       <c r="D7" s="8">
         <f>C7-B7</f>
@@ -1083,11 +1761,13 @@
           <t>Sous-traitance / freelances</t>
         </is>
       </c>
-      <c r="B8" s="11" t="n">
-        <v>24000</v>
-      </c>
-      <c r="C8" s="11" t="n">
-        <v>31000</v>
+      <c r="B8" s="11">
+        <f>Janvier!B8+Fevrier!B8+Mars!B8</f>
+        <v/>
+      </c>
+      <c r="C8" s="11">
+        <f>Janvier!C8+Fevrier!C8+Mars!C8</f>
+        <v/>
       </c>
       <c r="D8" s="11">
         <f>C8-B8</f>
@@ -1104,11 +1784,13 @@
           <t>Loyer et charges locatives</t>
         </is>
       </c>
-      <c r="B9" s="8" t="n">
-        <v>13500</v>
-      </c>
-      <c r="C9" s="8" t="n">
-        <v>13500</v>
+      <c r="B9" s="8">
+        <f>Janvier!B9+Fevrier!B9+Mars!B9</f>
+        <v/>
+      </c>
+      <c r="C9" s="8">
+        <f>Janvier!C9+Fevrier!C9+Mars!C9</f>
+        <v/>
       </c>
       <c r="D9" s="8">
         <f>C9-B9</f>
@@ -1125,11 +1807,13 @@
           <t>Marketing et acquisition</t>
         </is>
       </c>
-      <c r="B10" s="11" t="n">
-        <v>9000</v>
-      </c>
-      <c r="C10" s="11" t="n">
-        <v>11500</v>
+      <c r="B10" s="11">
+        <f>Janvier!B10+Fevrier!B10+Mars!B10</f>
+        <v/>
+      </c>
+      <c r="C10" s="11">
+        <f>Janvier!C10+Fevrier!C10+Mars!C10</f>
+        <v/>
       </c>
       <c r="D10" s="11">
         <f>C10-B10</f>
@@ -1146,11 +1830,13 @@
           <t>Informatique / outils</t>
         </is>
       </c>
-      <c r="B11" s="8" t="n">
-        <v>5400</v>
-      </c>
-      <c r="C11" s="8" t="n">
-        <v>5100</v>
+      <c r="B11" s="8">
+        <f>Janvier!B11+Fevrier!B11+Mars!B11</f>
+        <v/>
+      </c>
+      <c r="C11" s="8">
+        <f>Janvier!C11+Fevrier!C11+Mars!C11</f>
+        <v/>
       </c>
       <c r="D11" s="8">
         <f>C11-B11</f>
@@ -1167,11 +1853,13 @@
           <t>Autres frais généraux</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n">
-        <v>8100</v>
-      </c>
-      <c r="C12" s="11" t="n">
-        <v>7800</v>
+      <c r="B12" s="11">
+        <f>Janvier!B12+Fevrier!B12+Mars!B12</f>
+        <v/>
+      </c>
+      <c r="C12" s="11">
+        <f>Janvier!C12+Fevrier!C12+Mars!C12</f>
+        <v/>
       </c>
       <c r="D12" s="11">
         <f>C12-B12</f>
@@ -1251,21 +1939,37 @@
         <v/>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Contrôle</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="16" t="inlineStr">
+        <is>
+          <t>Chaque ligne Budget / Réalisé est la somme des trois feuilles mensuelles. Ex. CA honoraires Q1 : budget 280'000 | réalisé 251'000.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20"/>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
+    <mergeCell ref="A19:E20"/>
     <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
@@ -1365,14 +2069,30 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="18" t="inlineStr">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Cohérence trimestre</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Janvier + Février + Mars = Trimestre. Q1 CA : 280'000 budget / 251'000 réalisé (écart −29'000). Le trou se creuse surtout en mars (−18'000) après un février déjà faible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23"/>
+    <row r="25">
+      <c r="A25" s="18" t="inlineStr">
         <is>
           <t>Ne montrez pas cette feuille aux participants avant la fin de l'exercice.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
+    <mergeCell ref="A22:B23"/>
     <mergeCell ref="A4:B6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>